<commit_message>
lookup functions and error handling
</commit_message>
<xml_diff>
--- a/02_Wrangling.xlsx
+++ b/02_Wrangling.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f595840ab58673e5/Desktop/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_8CB69184ADCF9C0F8A1DF75E7B2DA5884B1E3251" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{2EC39B2F-004B-4492-B199-AA3D9CD4FD04}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_8CB69184ADCF9C0F8A1DF75E7B2DA5884B1E3251" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{1BBB8A61-BADF-48F6-BEE1-961745C59EA7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EmployeeData" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">EmployeeData!$A$10:$O$16</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="59">
   <si>
     <t>Full Name</t>
   </si>
@@ -273,10 +276,10 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -617,7 +620,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
@@ -816,10 +819,10 @@
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="3"/>
       <c r="E10" t="s">
         <v>53</v>
       </c>
@@ -832,19 +835,19 @@
       <c r="H10" t="s">
         <v>56</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3" t="s">
+      <c r="J10" s="4"/>
+      <c r="K10" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3" t="s">
+      <c r="L10" s="4"/>
+      <c r="M10" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -953,19 +956,19 @@
         <v>15</v>
       </c>
       <c r="E13" t="str">
-        <f t="shared" ref="E13:E16" si="0">PROPER(A13)</f>
+        <f>PROPER(A13)</f>
         <v>Jane Smith</v>
       </c>
       <c r="F13" t="str">
-        <f t="shared" ref="F13:F16" si="1">LOWER(D13)</f>
+        <f t="shared" ref="F13:F16" si="0">LOWER(D13)</f>
         <v>jane@example.com</v>
       </c>
       <c r="G13" t="str">
-        <f t="shared" ref="G13:G16" si="2">LEFT(A13,3)</f>
+        <f>LEFT(A13,3)</f>
         <v>jan</v>
       </c>
       <c r="H13" t="str">
-        <f t="shared" ref="H13:H16" si="3">MID(D13,2,7)</f>
+        <f t="shared" ref="H13:H16" si="1">MID(D13,2,7)</f>
         <v>ane@exa</v>
       </c>
       <c r="I13" t="s">
@@ -1005,19 +1008,19 @@
         <v>16</v>
       </c>
       <c r="E14" t="str">
+        <f>PROPER(A14)</f>
+        <v>Alice Johnson</v>
+      </c>
+      <c r="F14" t="str">
         <f t="shared" si="0"/>
-        <v>Alice Johnson</v>
-      </c>
-      <c r="F14" t="str">
+        <v>alice@example.com</v>
+      </c>
+      <c r="G14" t="str">
+        <f>LEFT(A14,3)</f>
+        <v>ALI</v>
+      </c>
+      <c r="H14" t="str">
         <f t="shared" si="1"/>
-        <v>alice@example.com</v>
-      </c>
-      <c r="G14" t="str">
-        <f t="shared" si="2"/>
-        <v>ALI</v>
-      </c>
-      <c r="H14" t="str">
-        <f t="shared" si="3"/>
         <v>lice@ex</v>
       </c>
       <c r="I14" t="s">
@@ -1057,19 +1060,19 @@
         <v>22</v>
       </c>
       <c r="E15" t="str">
+        <f>PROPER(A15)</f>
+        <v>Bob Brown</v>
+      </c>
+      <c r="F15" t="str">
         <f t="shared" si="0"/>
-        <v>Bob Brown</v>
-      </c>
-      <c r="F15" t="str">
+        <v>bob@example.com</v>
+      </c>
+      <c r="G15" t="str">
+        <f>LEFT(A15,3)</f>
+        <v>BOB</v>
+      </c>
+      <c r="H15" t="str">
         <f t="shared" si="1"/>
-        <v>bob@example.com</v>
-      </c>
-      <c r="G15" t="str">
-        <f t="shared" si="2"/>
-        <v>BOB</v>
-      </c>
-      <c r="H15" t="str">
-        <f t="shared" si="3"/>
         <v>OB@exam</v>
       </c>
       <c r="I15" t="s">
@@ -1084,15 +1087,12 @@
       <c r="L15" t="s">
         <v>41</v>
       </c>
-      <c r="M15" t="s">
-        <v>32</v>
-      </c>
       <c r="N15" t="s">
         <v>48</v>
       </c>
       <c r="O15" t="str">
-        <f t="shared" ref="O15:O16" si="4">_xlfn.TEXTJOIN("-",TRUE,M15,N15)</f>
-        <v>BOB-Brown</v>
+        <f t="shared" ref="O15:O16" si="2">_xlfn.TEXTJOIN("-",TRUE,M15,N15)</f>
+        <v>Brown</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
@@ -1109,19 +1109,19 @@
         <v>17</v>
       </c>
       <c r="E16" t="str">
+        <f>PROPER(A16)</f>
+        <v>Eva White</v>
+      </c>
+      <c r="F16" t="str">
         <f t="shared" si="0"/>
-        <v>Eva White</v>
-      </c>
-      <c r="F16" t="str">
+        <v>eva@example.com</v>
+      </c>
+      <c r="G16" t="str">
+        <f>LEFT(A16,3)</f>
+        <v>Eva</v>
+      </c>
+      <c r="H16" t="str">
         <f t="shared" si="1"/>
-        <v>eva@example.com</v>
-      </c>
-      <c r="G16" t="str">
-        <f t="shared" si="2"/>
-        <v>Eva</v>
-      </c>
-      <c r="H16" t="str">
-        <f t="shared" si="3"/>
         <v>va@exam</v>
       </c>
       <c r="I16" t="s">
@@ -1136,15 +1136,12 @@
       <c r="L16" t="s">
         <v>41</v>
       </c>
-      <c r="M16" t="s">
-        <v>49</v>
-      </c>
       <c r="N16" t="s">
         <v>50</v>
       </c>
       <c r="O16" t="str">
-        <f t="shared" si="4"/>
-        <v>Eva-White</v>
+        <f>_xlfn.TEXTJOIN("-",FALSE,M16,N16)</f>
+        <v>-White</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -1224,10 +1221,15 @@
         <v>45000</v>
       </c>
     </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1"/>
+    </row>
   </sheetData>
   <dataConsolidate leftLabels="1" topLabels="1">
-    <dataRefs count="1">
+    <dataRefs count="2">
       <dataRef ref="A21:B26" sheet="EmployeeData"/>
+      <dataRef ref="A38:B43" sheet="EmployeeData"/>
     </dataRefs>
   </dataConsolidate>
   <mergeCells count="4">

</xml_diff>